<commit_message>
Winamax Spanish Circuit 2026 Playoffs
</commit_message>
<xml_diff>
--- a/file/finances_updated.xlsx
+++ b/file/finances_updated.xlsx
@@ -755,7 +755,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C13">
-        <v>28500</v>
+        <v>29400</v>
       </c>
       <c r="D13">
         <v>500</v>
@@ -1074,7 +1074,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C24">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D24">
         <v>500</v>
@@ -1364,7 +1364,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C34">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D34">
         <v>500</v>
@@ -1567,7 +1567,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C41">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D41">
         <v>500</v>
@@ -1944,7 +1944,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C54">
-        <v>28500</v>
+        <v>30300</v>
       </c>
       <c r="D54">
         <v>500</v>
@@ -4264,7 +4264,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C134">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D134">
         <v>500</v>
@@ -5018,7 +5018,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C160">
-        <v>28500</v>
+        <v>29700</v>
       </c>
       <c r="D160">
         <v>500</v>
@@ -5105,7 +5105,7 @@
         <v>Tier 3</v>
       </c>
       <c r="C163">
-        <v>28500</v>
+        <v>28920</v>
       </c>
       <c r="D163">
         <v>500</v>

</xml_diff>